<commit_message>
fix: replace PwC with NGC as source in controls library
</commit_message>
<xml_diff>
--- a/docs/ngc_controls.xlsx
+++ b/docs/ngc_controls.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="14880" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NGC Controls" sheetId="1" state="visible" r:id="rId1"/>
@@ -13,7 +12,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NGC Controls'!$A$1:$G$39</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -31,13 +30,13 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001E3A5F"/>
+      <color rgb="FF1E3A5F"/>
       <sz val="9"/>
     </font>
     <font>
@@ -47,19 +46,19 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001D4ED8"/>
+      <color rgb="FF1D4ED8"/>
       <sz val="8"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="007C3AED"/>
+      <color rgb="FF7C3AED"/>
       <sz val="8"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00166534"/>
+      <color rgb="FF166534"/>
       <sz val="8"/>
     </font>
   </fonts>
@@ -72,27 +71,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E3A5F"/>
+        <fgColor rgb="FF1E3A5F"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EFF6FF"/>
+        <fgColor rgb="FFEFF6FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8FAFC"/>
+        <fgColor rgb="FFF8FAFC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F0FDF4"/>
+        <fgColor rgb="FFF0FDF4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -106,17 +105,18 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D1D5DB"/>
+        <color rgb="FFD1D5DB"/>
       </left>
       <right style="thin">
-        <color rgb="00D1D5DB"/>
+        <color rgb="FFD1D5DB"/>
       </right>
       <top style="thin">
-        <color rgb="00D1D5DB"/>
+        <color rgb="FFD1D5DB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D1D5DB"/>
+        <color rgb="FFD1D5DB"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -177,7 +177,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -543,12 +543,10 @@
   <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="5" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -622,7 +620,7 @@
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -659,7 +657,7 @@
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -696,7 +694,7 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -733,7 +731,7 @@
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -770,7 +768,7 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -807,7 +805,7 @@
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -844,7 +842,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -881,7 +879,7 @@
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -918,7 +916,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -955,7 +953,7 @@
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -992,7 +990,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1027,7 @@
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1064,7 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1101,7 @@
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1140,7 +1138,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1175,7 @@
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1212,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1249,7 @@
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1288,7 +1286,7 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1323,7 @@
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1362,7 +1360,7 @@
       </c>
       <c r="G22" s="13" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1397,7 @@
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1434,7 @@
       </c>
       <c r="G24" s="13" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1471,7 @@
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1508,7 @@
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1547,7 +1545,7 @@
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1584,7 +1582,7 @@
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1619,7 @@
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1658,7 +1656,7 @@
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1695,7 +1693,7 @@
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1730,7 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1769,7 +1767,7 @@
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1806,7 +1804,7 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1843,7 +1841,7 @@
       </c>
       <c r="G35" s="8" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1878,7 @@
       </c>
       <c r="G36" s="13" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1917,7 +1915,7 @@
       </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1954,7 +1952,7 @@
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>
@@ -1991,7 +1989,7 @@
       </c>
       <c r="G39" s="8" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>NGC</t>
         </is>
       </c>
     </row>

</xml_diff>